<commit_message>
Changed the freshmart dashboard based on brd
</commit_message>
<xml_diff>
--- a/Excel/Practice_files_lms/DA_BI_Practice_m8.xlsx
+++ b/Excel/Practice_files_lms/DA_BI_Practice_m8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rithiha\Excel\Practice_files_lms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D6E000-4EF2-46A2-8A4F-210AF7451E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5DFA06-CC95-46BE-A357-960923AA5424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1062,7 +1062,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1213,97 +1213,96 @@
     <xf numFmtId="10" fontId="15" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1531,25 +1530,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="56"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="70"/>
     </row>
     <row r="2" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="56"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="70"/>
     </row>
     <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="56"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1597,11 +1596,11 @@
       </c>
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="67" t="s">
+      <c r="A11" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="56"/>
+      <c r="B11" s="69"/>
+      <c r="C11" s="70"/>
     </row>
     <row r="12" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
@@ -2655,49 +2654,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="56"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="70"/>
     </row>
     <row r="2" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="56"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="70"/>
     </row>
     <row r="4" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="56"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="70"/>
     </row>
     <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="56"/>
-      <c r="E5" s="58" t="s">
+      <c r="B5" s="69"/>
+      <c r="C5" s="70"/>
+      <c r="E5" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="55"/>
-      <c r="G5" s="56"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="70"/>
     </row>
     <row r="6" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
@@ -2721,11 +2720,11 @@
       <c r="B7" s="22">
         <v>3.0704170642958762E-2</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="87" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="70"/>
     </row>
     <row r="8" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
@@ -2734,97 +2733,97 @@
       <c r="B8" s="23">
         <v>60</v>
       </c>
-      <c r="E8" s="63" t="s">
+      <c r="E8" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="55"/>
-      <c r="G8" s="56"/>
+      <c r="F8" s="69"/>
+      <c r="G8" s="70"/>
     </row>
     <row r="10" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="56"/>
+      <c r="B10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="70"/>
     </row>
     <row r="11" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="55"/>
-      <c r="G11" s="56"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="70"/>
     </row>
     <row r="12" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="82" t="s">
         <v>160</v>
       </c>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="56"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="69"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="70"/>
     </row>
     <row r="13" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="54" t="s">
+      <c r="B13" s="82" t="s">
         <v>161</v>
       </c>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="55"/>
-      <c r="F13" s="55"/>
-      <c r="G13" s="56"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="70"/>
     </row>
     <row r="14" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="82" t="s">
         <v>162</v>
       </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="56"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="69"/>
+      <c r="G14" s="70"/>
     </row>
     <row r="16" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="61" t="s">
+      <c r="A16" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="56"/>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="70"/>
     </row>
     <row r="17" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="62" t="s">
+      <c r="A17" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="55"/>
-      <c r="C17" s="56"/>
-      <c r="E17" s="58" t="s">
+      <c r="B17" s="69"/>
+      <c r="C17" s="70"/>
+      <c r="E17" s="74" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="55"/>
-      <c r="G17" s="56"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="70"/>
     </row>
     <row r="18" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
@@ -2882,79 +2881,79 @@
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="59" t="s">
+      <c r="A23" s="75" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="56"/>
+      <c r="B23" s="69"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="69"/>
+      <c r="G23" s="70"/>
     </row>
     <row r="24" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="82" t="s">
         <v>163</v>
       </c>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="56"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="70"/>
     </row>
     <row r="25" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="54" t="s">
+      <c r="B25" s="82" t="s">
         <v>164</v>
       </c>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="56"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="70"/>
     </row>
     <row r="26" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="82" t="s">
         <v>165</v>
       </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56"/>
+      <c r="C26" s="69"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="69"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="70"/>
     </row>
     <row r="27" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="54" t="s">
+      <c r="B27" s="82" t="s">
         <v>166</v>
       </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="56"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="70"/>
     </row>
     <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="60" t="s">
+      <c r="A29" s="76" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="56"/>
+      <c r="B29" s="69"/>
+      <c r="C29" s="69"/>
+      <c r="D29" s="69"/>
+      <c r="E29" s="69"/>
+      <c r="F29" s="69"/>
+      <c r="G29" s="70"/>
     </row>
     <row r="30" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
@@ -2980,66 +2979,66 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="59" t="s">
+      <c r="A32" s="75" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="55"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="56"/>
+      <c r="B32" s="69"/>
+      <c r="C32" s="69"/>
+      <c r="D32" s="69"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="69"/>
+      <c r="G32" s="70"/>
     </row>
     <row r="33" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="54" t="s">
+      <c r="B33" s="82" t="s">
         <v>167</v>
       </c>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="56"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="69"/>
+      <c r="E33" s="69"/>
+      <c r="F33" s="69"/>
+      <c r="G33" s="70"/>
     </row>
     <row r="34" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="54" t="s">
+      <c r="B34" s="82" t="s">
         <v>168</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="56"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="69"/>
+      <c r="G34" s="70"/>
     </row>
     <row r="35" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="54" t="s">
+      <c r="B35" s="82" t="s">
         <v>169</v>
       </c>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="56"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="69"/>
+      <c r="E35" s="69"/>
+      <c r="F35" s="69"/>
+      <c r="G35" s="70"/>
     </row>
     <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="57" t="s">
+      <c r="A37" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="56"/>
+      <c r="B37" s="69"/>
+      <c r="C37" s="69"/>
+      <c r="D37" s="69"/>
+      <c r="E37" s="69"/>
+      <c r="F37" s="69"/>
+      <c r="G37" s="70"/>
     </row>
     <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4006,21 +4005,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A32:G32"/>
     <mergeCell ref="B33:G33"/>
     <mergeCell ref="B34:G34"/>
     <mergeCell ref="B35:G35"/>
@@ -4032,6 +4016,21 @@
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="A29:G29"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="E5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4049,43 +4048,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="68" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="70"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="56"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="70"/>
     </row>
     <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="72" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="56"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
     </row>
     <row r="5" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
@@ -4109,13 +4108,13 @@
       <c r="B6" s="22">
         <v>0.1</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="87" t="s">
         <v>70</v>
       </c>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="56"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="70"/>
     </row>
     <row r="7" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
@@ -4126,30 +4125,30 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="88" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="55"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="56"/>
+      <c r="B9" s="69"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="69"/>
+      <c r="H9" s="69"/>
+      <c r="I9" s="70"/>
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="83" t="s">
         <v>72</v>
       </c>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="56"/>
+      <c r="B10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="70"/>
     </row>
     <row r="11" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="16" t="s">
@@ -4165,7 +4164,7 @@
         <v>0.08</v>
       </c>
       <c r="D12" s="30">
-        <f t="dataTable" ref="D12:D18" dt2D="0" dtr="0" r1="B6"/>
+        <f t="dataTable" ref="D12:D18" dt2D="0" dtr="0" r1="B6" ca="1"/>
         <v>10138.197144206841</v>
       </c>
     </row>
@@ -4218,43 +4217,43 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="56"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="69"/>
+      <c r="H19" s="69"/>
+      <c r="I19" s="70"/>
     </row>
     <row r="21" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="61" t="s">
+      <c r="A21" s="88" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="55"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="56"/>
+      <c r="B21" s="69"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="69"/>
+      <c r="H21" s="69"/>
+      <c r="I21" s="70"/>
     </row>
     <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="68" t="s">
+      <c r="A22" s="83" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="55"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="56"/>
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="69"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
+      <c r="I22" s="70"/>
     </row>
     <row r="23" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F23" s="16" t="s">
@@ -4270,7 +4269,7 @@
         <v>200000</v>
       </c>
       <c r="G24" s="30">
-        <f t="dataTable" ref="G24:G32" dt2D="0" dtr="0" r1="B5" ca="1"/>
+        <f t="dataTable" ref="G24:G32" dt2D="0" dtr="0" r1="B5"/>
         <v>4249.4089422536554</v>
       </c>
     </row>
@@ -4340,17 +4339,17 @@
     </row>
     <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="72" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="55"/>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="56"/>
+      <c r="B34" s="69"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="69"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="70"/>
     </row>
     <row r="35" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="19" t="s">
@@ -4385,30 +4384,30 @@
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="59" t="s">
+      <c r="A39" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="B39" s="55"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55"/>
-      <c r="H39" s="55"/>
-      <c r="I39" s="56"/>
+      <c r="B39" s="69"/>
+      <c r="C39" s="69"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="69"/>
+      <c r="F39" s="69"/>
+      <c r="G39" s="69"/>
+      <c r="H39" s="69"/>
+      <c r="I39" s="70"/>
     </row>
     <row r="40" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="68" t="s">
+      <c r="A40" s="83" t="s">
         <v>79</v>
       </c>
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="56"/>
+      <c r="B40" s="69"/>
+      <c r="C40" s="69"/>
+      <c r="D40" s="69"/>
+      <c r="E40" s="69"/>
+      <c r="F40" s="69"/>
+      <c r="G40" s="69"/>
+      <c r="H40" s="69"/>
+      <c r="I40" s="70"/>
     </row>
     <row r="41" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="33">
@@ -4534,120 +4533,120 @@
     </row>
     <row r="47" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="68" t="s">
+      <c r="A48" s="83" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="55"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="56"/>
+      <c r="B48" s="69"/>
+      <c r="C48" s="69"/>
+      <c r="D48" s="69"/>
+      <c r="E48" s="69"/>
+      <c r="F48" s="69"/>
+      <c r="G48" s="69"/>
+      <c r="H48" s="69"/>
+      <c r="I48" s="70"/>
     </row>
     <row r="49" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="69" t="s">
+      <c r="A50" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="55"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="55"/>
-      <c r="F50" s="55"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
+      <c r="B50" s="69"/>
+      <c r="C50" s="69"/>
+      <c r="D50" s="69"/>
+      <c r="E50" s="69"/>
+      <c r="F50" s="69"/>
+      <c r="G50" s="69"/>
+      <c r="H50" s="69"/>
+      <c r="I50" s="70"/>
     </row>
     <row r="51" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B51" s="54" t="s">
+      <c r="B51" s="82" t="s">
         <v>174</v>
       </c>
-      <c r="C51" s="55"/>
-      <c r="D51" s="55"/>
-      <c r="E51" s="55"/>
-      <c r="F51" s="55"/>
-      <c r="G51" s="55"/>
-      <c r="H51" s="55"/>
-      <c r="I51" s="56"/>
+      <c r="C51" s="69"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="69"/>
+      <c r="F51" s="69"/>
+      <c r="G51" s="69"/>
+      <c r="H51" s="69"/>
+      <c r="I51" s="70"/>
     </row>
     <row r="52" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B52" s="54" t="s">
+      <c r="B52" s="82" t="s">
         <v>173</v>
       </c>
-      <c r="C52" s="55"/>
-      <c r="D52" s="55"/>
-      <c r="E52" s="55"/>
-      <c r="F52" s="55"/>
-      <c r="G52" s="55"/>
-      <c r="H52" s="55"/>
-      <c r="I52" s="56"/>
+      <c r="C52" s="69"/>
+      <c r="D52" s="69"/>
+      <c r="E52" s="69"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="69"/>
+      <c r="H52" s="69"/>
+      <c r="I52" s="70"/>
     </row>
     <row r="53" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="B53" s="54" t="s">
+      <c r="B53" s="82" t="s">
         <v>170</v>
       </c>
-      <c r="C53" s="55"/>
-      <c r="D53" s="55"/>
-      <c r="E53" s="55"/>
-      <c r="F53" s="55"/>
-      <c r="G53" s="55"/>
-      <c r="H53" s="55"/>
-      <c r="I53" s="56"/>
+      <c r="C53" s="69"/>
+      <c r="D53" s="69"/>
+      <c r="E53" s="69"/>
+      <c r="F53" s="69"/>
+      <c r="G53" s="69"/>
+      <c r="H53" s="69"/>
+      <c r="I53" s="70"/>
     </row>
     <row r="54" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B54" s="54" t="s">
+      <c r="B54" s="82" t="s">
         <v>172</v>
       </c>
-      <c r="C54" s="55"/>
-      <c r="D54" s="55"/>
-      <c r="E54" s="55"/>
-      <c r="F54" s="55"/>
-      <c r="G54" s="55"/>
-      <c r="H54" s="55"/>
-      <c r="I54" s="56"/>
+      <c r="C54" s="69"/>
+      <c r="D54" s="69"/>
+      <c r="E54" s="69"/>
+      <c r="F54" s="69"/>
+      <c r="G54" s="69"/>
+      <c r="H54" s="69"/>
+      <c r="I54" s="70"/>
     </row>
     <row r="55" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B55" s="54" t="s">
+      <c r="B55" s="82" t="s">
         <v>171</v>
       </c>
-      <c r="C55" s="55"/>
-      <c r="D55" s="55"/>
-      <c r="E55" s="55"/>
-      <c r="F55" s="55"/>
-      <c r="G55" s="55"/>
-      <c r="H55" s="55"/>
-      <c r="I55" s="56"/>
+      <c r="C55" s="69"/>
+      <c r="D55" s="69"/>
+      <c r="E55" s="69"/>
+      <c r="F55" s="69"/>
+      <c r="G55" s="69"/>
+      <c r="H55" s="69"/>
+      <c r="I55" s="70"/>
     </row>
     <row r="56" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="57" t="s">
+      <c r="A57" s="84" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="55"/>
-      <c r="C57" s="55"/>
-      <c r="D57" s="55"/>
-      <c r="E57" s="55"/>
-      <c r="F57" s="55"/>
-      <c r="G57" s="55"/>
-      <c r="H57" s="55"/>
-      <c r="I57" s="56"/>
+      <c r="B57" s="69"/>
+      <c r="C57" s="69"/>
+      <c r="D57" s="69"/>
+      <c r="E57" s="69"/>
+      <c r="F57" s="69"/>
+      <c r="G57" s="69"/>
+      <c r="H57" s="69"/>
+      <c r="I57" s="70"/>
     </row>
     <row r="58" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5594,16 +5593,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B54:I54"/>
     <mergeCell ref="B55:I55"/>
     <mergeCell ref="A57:I57"/>
@@ -5614,6 +5603,16 @@
     <mergeCell ref="A40:I40"/>
     <mergeCell ref="A48:I48"/>
     <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A9:I9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -5634,152 +5633,151 @@
   <sheetData>
     <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="57" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" collapsed="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="83" t="s">
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="63" t="s">
         <v>181</v>
       </c>
-      <c r="E3" s="83" t="s">
+      <c r="E3" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="F3" s="83" t="s">
+      <c r="F3" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="G3" s="83" t="s">
+      <c r="G3" s="63" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="22.5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="86" t="s">
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="E4" s="66" t="s">
         <v>178</v>
       </c>
-      <c r="F4" s="86" t="s">
+      <c r="F4" s="66" t="s">
         <v>178</v>
       </c>
-      <c r="G4" s="86" t="s">
+      <c r="G4" s="66" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="80" t="s">
+      <c r="B5" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="C5" s="80"/>
-      <c r="D5" s="78"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="78"/>
-      <c r="G5" s="78"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
     </row>
     <row r="6" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="79"/>
-      <c r="C6" s="79" t="s">
+      <c r="B6" s="59"/>
+      <c r="C6" s="59" t="s">
         <v>175</v>
       </c>
-      <c r="D6" s="74">
+      <c r="D6" s="54">
         <v>1800000</v>
       </c>
-      <c r="E6" s="84">
+      <c r="E6" s="64">
         <v>800000</v>
       </c>
-      <c r="F6" s="84">
+      <c r="F6" s="64">
         <v>1200000</v>
       </c>
-      <c r="G6" s="84">
+      <c r="G6" s="64">
         <v>1800000</v>
       </c>
     </row>
     <row r="7" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="79"/>
-      <c r="C7" s="79" t="s">
+      <c r="B7" s="59"/>
+      <c r="C7" s="59" t="s">
         <v>176</v>
       </c>
-      <c r="D7" s="74">
+      <c r="D7" s="54">
         <v>900000</v>
       </c>
-      <c r="E7" s="84">
+      <c r="E7" s="64">
         <v>750000</v>
       </c>
-      <c r="F7" s="84">
+      <c r="F7" s="64">
         <v>800000</v>
       </c>
-      <c r="G7" s="84">
+      <c r="G7" s="64">
         <v>900000</v>
       </c>
     </row>
     <row r="8" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="79"/>
-      <c r="C8" s="79" t="s">
+      <c r="B8" s="59"/>
+      <c r="C8" s="59" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="75">
+      <c r="D8" s="55">
         <v>0.25</v>
       </c>
-      <c r="E8" s="85">
+      <c r="E8" s="65">
         <v>0.3</v>
       </c>
-      <c r="F8" s="85">
+      <c r="F8" s="65">
         <v>0.28000000000000003</v>
       </c>
-      <c r="G8" s="85">
+      <c r="G8" s="65">
         <v>0.25</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="80" t="s">
+      <c r="B9" s="60" t="s">
         <v>182</v>
       </c>
-      <c r="C9" s="80"/>
-      <c r="D9" s="78"/>
-      <c r="E9" s="78"/>
-      <c r="F9" s="78"/>
-      <c r="G9" s="78"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
     </row>
     <row r="10" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="79"/>
-      <c r="C10" s="79" t="s">
+      <c r="B10" s="59"/>
+      <c r="C10" s="59" t="s">
         <v>187</v>
       </c>
-      <c r="D10" s="74">
+      <c r="D10" s="54">
         <v>675000</v>
       </c>
-      <c r="E10" s="74">
+      <c r="E10" s="54">
         <v>35000</v>
       </c>
-      <c r="F10" s="74">
+      <c r="F10" s="54">
         <v>288000</v>
       </c>
-      <c r="G10" s="74">
+      <c r="G10" s="54">
         <v>675000</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="81"/>
-      <c r="C11" s="81" t="s">
+      <c r="B11" s="61"/>
+      <c r="C11" s="61" t="s">
         <v>188</v>
       </c>
-      <c r="D11" s="88">
+      <c r="D11" s="67">
         <v>0.375</v>
       </c>
-      <c r="E11" s="88">
+      <c r="E11" s="67">
         <v>4.3749999999999997E-2</v>
       </c>
-      <c r="F11" s="88">
+      <c r="F11" s="67">
         <v>0.24</v>
       </c>
-      <c r="G11" s="88">
+      <c r="G11" s="67">
         <v>0.375</v>
       </c>
     </row>
@@ -5820,48 +5818,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="56"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="70"/>
     </row>
     <row r="2" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="56"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="70"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="72" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="70"/>
     </row>
     <row r="5" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="56"/>
+      <c r="B5" s="70"/>
     </row>
     <row r="6" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
@@ -5888,10 +5886,10 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="56"/>
+      <c r="B10" s="70"/>
     </row>
     <row r="11" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
@@ -5930,18 +5928,18 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="75" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="56"/>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="69"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="70"/>
     </row>
     <row r="17" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
@@ -6023,18 +6021,18 @@
     </row>
     <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="60" t="s">
+      <c r="A22" s="76" t="s">
         <v>108</v>
       </c>
-      <c r="B22" s="55"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="56"/>
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="69"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
+      <c r="I22" s="69"/>
+      <c r="J22" s="70"/>
     </row>
     <row r="23" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45" t="s">
@@ -6117,257 +6115,257 @@
       </c>
     </row>
     <row r="27" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="72" t="s">
         <v>122</v>
       </c>
-      <c r="B27" s="55"/>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="55"/>
-      <c r="H27" s="55"/>
-      <c r="I27" s="55"/>
-      <c r="J27" s="56"/>
+      <c r="B27" s="69"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="69"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="69"/>
+      <c r="J27" s="70"/>
     </row>
     <row r="28" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="B28" s="71" t="s">
+      <c r="B28" s="77" t="s">
         <v>124</v>
       </c>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="56"/>
+      <c r="C28" s="69"/>
+      <c r="D28" s="69"/>
+      <c r="E28" s="69"/>
+      <c r="F28" s="70"/>
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="B29" s="72" t="s">
+      <c r="B29" s="78" t="s">
         <v>126</v>
       </c>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="56"/>
+      <c r="C29" s="69"/>
+      <c r="D29" s="69"/>
+      <c r="E29" s="69"/>
+      <c r="F29" s="70"/>
     </row>
     <row r="30" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="B30" s="71" t="s">
+      <c r="B30" s="77" t="s">
         <v>128</v>
       </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="56"/>
+      <c r="C30" s="69"/>
+      <c r="D30" s="69"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="70"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="89" t="s">
+      <c r="B31" s="79" t="s">
         <v>130</v>
       </c>
-      <c r="C31" s="55"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="56"/>
+      <c r="C31" s="69"/>
+      <c r="D31" s="69"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="70"/>
     </row>
     <row r="32" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="B32" s="90" t="s">
+      <c r="B32" s="80" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="56"/>
+      <c r="C32" s="69"/>
+      <c r="D32" s="69"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="70"/>
     </row>
     <row r="33" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="89" t="s">
+      <c r="B33" s="79" t="s">
         <v>134</v>
       </c>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="56"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="69"/>
+      <c r="E33" s="69"/>
+      <c r="F33" s="70"/>
     </row>
     <row r="34" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="B34" s="71" t="s">
+      <c r="B34" s="77" t="s">
         <v>136</v>
       </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="56"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="70"/>
     </row>
     <row r="35" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="B35" s="72" t="s">
+      <c r="B35" s="78" t="s">
         <v>138</v>
       </c>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="56"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="69"/>
+      <c r="E35" s="69"/>
+      <c r="F35" s="70"/>
     </row>
     <row r="36" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="B36" s="71" t="s">
+      <c r="B36" s="77" t="s">
         <v>140</v>
       </c>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="56"/>
+      <c r="C36" s="69"/>
+      <c r="D36" s="69"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="70"/>
     </row>
     <row r="37" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="75" t="s">
         <v>141</v>
       </c>
-      <c r="B38" s="55"/>
-      <c r="C38" s="55"/>
-      <c r="D38" s="55"/>
-      <c r="E38" s="55"/>
-      <c r="F38" s="55"/>
-      <c r="G38" s="55"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="56"/>
+      <c r="B38" s="69"/>
+      <c r="C38" s="69"/>
+      <c r="D38" s="69"/>
+      <c r="E38" s="69"/>
+      <c r="F38" s="69"/>
+      <c r="G38" s="69"/>
+      <c r="H38" s="69"/>
+      <c r="I38" s="69"/>
+      <c r="J38" s="70"/>
     </row>
     <row r="39" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="B39" s="54" t="s">
+      <c r="B39" s="82" t="s">
         <v>143</v>
       </c>
-      <c r="C39" s="55"/>
-      <c r="D39" s="55"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="56"/>
+      <c r="C39" s="69"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="69"/>
+      <c r="F39" s="70"/>
     </row>
     <row r="40" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="87" t="s">
+      <c r="B40" s="81" t="s">
         <v>186</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="56"/>
+      <c r="C40" s="69"/>
+      <c r="D40" s="69"/>
+      <c r="E40" s="69"/>
+      <c r="F40" s="70"/>
     </row>
     <row r="41" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="B41" s="54" t="s">
+      <c r="B41" s="82" t="s">
         <v>146</v>
       </c>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="56"/>
+      <c r="C41" s="69"/>
+      <c r="D41" s="69"/>
+      <c r="E41" s="69"/>
+      <c r="F41" s="70"/>
     </row>
     <row r="42" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="B42" s="87" t="s">
+      <c r="B42" s="81" t="s">
         <v>189</v>
       </c>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="56"/>
+      <c r="C42" s="69"/>
+      <c r="D42" s="69"/>
+      <c r="E42" s="69"/>
+      <c r="F42" s="70"/>
     </row>
     <row r="43" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="B43" s="87" t="s">
+      <c r="B43" s="81" t="s">
         <v>149</v>
       </c>
-      <c r="C43" s="55"/>
-      <c r="D43" s="55"/>
-      <c r="E43" s="55"/>
-      <c r="F43" s="56"/>
+      <c r="C43" s="69"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="69"/>
+      <c r="F43" s="70"/>
     </row>
     <row r="44" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="B44" s="87" t="s">
+      <c r="B44" s="81" t="s">
         <v>190</v>
       </c>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="56"/>
+      <c r="C44" s="69"/>
+      <c r="D44" s="69"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="70"/>
     </row>
     <row r="45" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="68" t="s">
+      <c r="A46" s="83" t="s">
         <v>151</v>
       </c>
-      <c r="B46" s="55"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="55"/>
-      <c r="H46" s="55"/>
-      <c r="I46" s="55"/>
-      <c r="J46" s="56"/>
+      <c r="B46" s="69"/>
+      <c r="C46" s="69"/>
+      <c r="D46" s="69"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
+      <c r="G46" s="69"/>
+      <c r="H46" s="69"/>
+      <c r="I46" s="69"/>
+      <c r="J46" s="70"/>
     </row>
     <row r="47" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="57" t="s">
+      <c r="A47" s="84" t="s">
         <v>152</v>
       </c>
-      <c r="B47" s="55"/>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="55"/>
-      <c r="F47" s="55"/>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="55"/>
-      <c r="J47" s="56"/>
+      <c r="B47" s="69"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="69"/>
+      <c r="J47" s="70"/>
     </row>
     <row r="48" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="70" t="s">
+      <c r="A49" s="85" t="s">
         <v>153</v>
       </c>
-      <c r="B49" s="55"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="56"/>
+      <c r="B49" s="69"/>
+      <c r="C49" s="69"/>
+      <c r="D49" s="69"/>
+      <c r="E49" s="69"/>
+      <c r="F49" s="69"/>
+      <c r="G49" s="69"/>
+      <c r="H49" s="69"/>
+      <c r="I49" s="69"/>
+      <c r="J49" s="70"/>
     </row>
     <row r="50" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="37" t="s">
@@ -7439,16 +7437,11 @@
     </scenario>
   </scenarios>
   <mergeCells count="27">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A27:J27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A47:J47"/>
+    <mergeCell ref="A49:J49"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
@@ -7461,11 +7454,16 @@
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B41:F41"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A47:J47"/>
-    <mergeCell ref="A49:J49"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>